<commit_message>
change language to Persian
</commit_message>
<xml_diff>
--- a/data/Engineer_Room_1404_2.xlsx
+++ b/data/Engineer_Room_1404_2.xlsx
@@ -527,17 +527,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>احسان پور</t>
+          <t>نصیری</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>احسان پور</t>
+          <t>نصیری</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>احسان پور</t>
+          <t>نصیری</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>نصیری</t>
+          <t>احسان پور</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>نصیری</t>
+          <t>احسان پور</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>نصیری</t>
+          <t>احسان پور</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">

</xml_diff>